<commit_message>
Regenerate data with the Applitrack encoding fix applied
Supersedes c038c6b, which was committed before the Windows-1252
decoding bug (56061f8) was found and fixed. 10 districts that
previously showed 0 postings now show their real counts -- K-12 rows
go from 629 to 836. HE data is unchanged (that pipeline stage doesn't
use Applitrack). Verified against a live chromote render of every
affected district's actual page before treating this as correct.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Archived_HE_Data/hedata_2026-08-03.xlsx
+++ b/Archived_HE_Data/hedata_2026-08-03.xlsx
@@ -1986,7 +1986,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Part-time Faculty Pool - Construction Instructor</t>
+          <t>Part-time Faculty Pool - English Instructor</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2025-06-03</t>
+          <t>2021-10-14</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4099</t>
+          <t>https://jobs.sheridan.edu/postings/2725</t>
         </is>
       </c>
       <c r="F55" s="2">
@@ -2016,7 +2016,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Part-time Faculty Pool - English Instructor</t>
+          <t>Hospitality Faculty Coordinator</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2021-10-14</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/2725</t>
+          <t>https://jobs.sheridan.edu/postings/4660</t>
         </is>
       </c>
       <c r="F56" s="2">
@@ -2046,7 +2046,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Hospitality Faculty Coordinator</t>
+          <t>Part-time Faculty Pool - Construction Instructor</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2025-06-03</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4660</t>
+          <t>https://jobs.sheridan.edu/postings/4099</t>
         </is>
       </c>
       <c r="F57" s="2">
@@ -2376,7 +2376,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Residential Life Coordinator</t>
+          <t>Part-time Faculty Pool - Online Criminal Justice Instructor</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2025-06-03</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4568</t>
+          <t>https://jobs.sheridan.edu/postings/4086</t>
         </is>
       </c>
       <c r="F68" s="2">
@@ -2406,7 +2406,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Part-time Faculty Pool - Online Criminal Justice Instructor</t>
+          <t>Residential Life Coordinator</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2025-06-03</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4086</t>
+          <t>https://jobs.sheridan.edu/postings/4568</t>
         </is>
       </c>
       <c r="F69" s="2">
@@ -2796,7 +2796,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Part-time Faculty Pool - Math Instructor</t>
+          <t>(Student Position) WCA Gallery Assistant</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2024-09-27</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/3938</t>
+          <t>https://jobs.sheridan.edu/postings/4507</t>
         </is>
       </c>
       <c r="F82" s="2">
@@ -2826,7 +2826,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>(Student Position) WCA Gallery Assistant</t>
+          <t>Part-time Faculty Pool - Math Instructor</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2024-09-27</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4507</t>
+          <t>https://jobs.sheridan.edu/postings/3938</t>
         </is>
       </c>
       <c r="F83" s="2">
@@ -2976,7 +2976,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Part-time Faculty Pool - History Instructor</t>
+          <t>Administrative &amp; Work Based Learning Coordinator</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2025-06-03</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4098</t>
+          <t>https://jobs.sheridan.edu/postings/4656</t>
         </is>
       </c>
       <c r="F88" s="2">
@@ -3006,7 +3006,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Administrative &amp; Work Based Learning Coordinator</t>
+          <t>Part-time Faculty Pool - History Instructor</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2025-06-03</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4656</t>
+          <t>https://jobs.sheridan.edu/postings/4098</t>
         </is>
       </c>
       <c r="F89" s="2">
@@ -3096,7 +3096,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Part-time Faculty Pool - Hospitality/Tourism</t>
+          <t>Part-time Faculty Pool - Dental Hygiene Instructor</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2025-06-03</t>
+          <t>2021-12-08</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4101</t>
+          <t>https://jobs.sheridan.edu/postings/2847</t>
         </is>
       </c>
       <c r="F92" s="2">
@@ -3126,7 +3126,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Part-time Faculty Pool - Dental Hygiene Instructor</t>
+          <t>Custodial Manager</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2021-12-08</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/2847</t>
+          <t>https://jobs.sheridan.edu/postings/4665</t>
         </is>
       </c>
       <c r="F93" s="2">
@@ -3156,7 +3156,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Custodial Manager</t>
+          <t>Part-time Faculty Pool - Hospitality/Tourism</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2025-06-03</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4665</t>
+          <t>https://jobs.sheridan.edu/postings/4101</t>
         </is>
       </c>
       <c r="F94" s="2">
@@ -3336,7 +3336,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>(Student Position) Box Office Assistant</t>
+          <t>Part-time Faculty Pool - Human Services Instructor</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2025-06-03</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4560</t>
+          <t>https://jobs.sheridan.edu/postings/4085</t>
         </is>
       </c>
       <c r="F100" s="2">
@@ -3366,7 +3366,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Part-time Faculty Pool - Human Services Instructor</t>
+          <t>(Student Position) Box Office Assistant</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2025-06-03</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4085</t>
+          <t>https://jobs.sheridan.edu/postings/4560</t>
         </is>
       </c>
       <c r="F101" s="2">
@@ -3756,7 +3756,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Part-time Faculty Pool - Agriculture Instructor</t>
+          <t>(Student Position) Information Technology (IT) Night Helpdesk</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2024-07-18</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/3852</t>
+          <t>https://jobs.sheridan.edu/postings/4502</t>
         </is>
       </c>
       <c r="F114" s="2">
@@ -3786,7 +3786,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>(Student Position) Information Technology (IT) Night Helpdesk</t>
+          <t>Part-time Faculty Pool - Agriculture Instructor</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2024-07-18</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://jobs.sheridan.edu/postings/4502</t>
+          <t>https://jobs.sheridan.edu/postings/3852</t>
         </is>
       </c>
       <c r="F115" s="2">

</xml_diff>